<commit_message>
Überarbeitung bis einschließlich "serielle Komunikation"
</commit_message>
<xml_diff>
--- a/Doc/StoffverteilungV3.xlsx
+++ b/Doc/StoffverteilungV3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marti\Documents\KI_Kurs\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A72A37F-4143-4CEA-A063-0E55139A4F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6103E6E-CE19-4082-B900-E3E0E81E39FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8239FEFA-D283-4303-90C1-2785058B5E4E}"/>
   </bookViews>
@@ -1788,141 +1788,6 @@
     <t>https://netron.app/</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Netron.app</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:
-Öffne die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Datei</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: trained_letter_S_F_Z_int8.tflite
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Input</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> und </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Output</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> anschauen, int8, Dimensionen, Softmax
-Öffne die Datei: trained_letter_S_F_Z_float32.lite
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Input</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> und </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Output</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> anschauen, float32, Dimensionen, Softmax</t>
-    </r>
-  </si>
-  <si>
     <t>KI-Modell verbessern</t>
   </si>
   <si>
@@ -2607,727 +2472,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Edge Impulse:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> In diesem Schritt passt du die Bildeinstellungen an und generierst die Merkmale aus den Eingabedaten. Merkmale sind eindeutige Eigenschaften, die vom Klassifizierungsalgorithmus verwendet werden, um die Objekte zu erkennen. (...) Navigieren im Menü unter „Impulse Design“ zum Punkt </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Image“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Stelle die Farbtiefe auf „RGB“ ein und </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>speichere die Parameter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.
-Klicke anschließend auf </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Generate Features“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Der Analysevorgang wird – abhängig von der Anzahl der hochgeladenen Bilder – einige Zeit in Anspruch nehmen.
-Sobald er abgeschlossen ist, kannst du die Ergebnisse begutachten. Im Feature Explorer siehst du eine Visualisierung der Merkmale. Du kannst erkennen, dass
-einige Buchstaben S  (orange Punkte) und Buchstaben F (blaue Punkte) nur schwer voneinander zu unterscheiden sind und sich daher einige Datenpunkte in unmittelbarer Nähe zueinander befinden. Der Buchstabe Z lässt sich leichter abgrenzen. (...)
-(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Edge Impulse:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Benutzername, E-Mail-Adresse, Passwort (merken !!), Bedingungen zustimmen, E-Mail empfangen, Account aktivieren -&gt; Welcome 
-Image Classification auswählen, Target OpenMV H7 Plus auswählen, Quit Tutorial
-Keys/ Add new API key: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Development Key </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Warnung</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ignorieren
-In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OpenMV IDE:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Extras/ Datensatzeditor/ </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Neuer Datensatz</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: Neuen
- Ordner letter_S_F_Z erstellen und auswählen
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bearbeite</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> das ereits geöffnete </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bildaufnahmeskript</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:
-Die Kamera steht auf dem Kopf. Füge deshalb hinter Zeile 12 ein: 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-      </rPr>
-      <t>sensor.set_vflip(True) # Flips the image vertically</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve">sensor.set_hmirror(True) # Mirrors the image horizontally
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">In der </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Werkzeugleiste</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: Klicke auf das Symbol </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Neuer Klassenordner</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">/ letter_S erstellen
-Führe nun das Bildaufnahmeskript aus, indem du die OpenMV IDE mit der Kamera </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>verbindest</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> auf die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wiedergabetaste</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> klickst. 
-Fokussiere den Buchstaben S mit der Kamera und klicke auf das Symbol </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Daten erfassen</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, um ein Bild davon aufzunehmen. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wiederhole</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> dies 30x. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ändere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Abstand und Winkel zwischen den Aufnahmen. 
-Ebenso: In der Werkzeugleiste ... letter_F ... Buchstabe F
-Ebenso: In der Werkzeugleiste ... letter_Z ... Buchstabe Z
-Ebenso: In der Werkzeugleiste ... unknown ... Buchstabe U oder leere Tafel
-(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Im</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Windows Datei-Explorer: 
-Entpacke</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Datei ei-&lt;user&gt;-&lt;project&gt;-openmv-v-&lt;number&gt;-impulse-#1.zip
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Benenne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Dateien </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>um</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:
-Vorher: trained.tflite  Nachher: trained_letter_S_F_Z_int8.tflite
-Vorher: labels.txt         Nachher: labels_letter_S_F_Z.txt
-Vorher: ei_image_classification.py 
-Nacher: ei_image_classification_letter_S_F_Z_int8.py
-Vorher: ei-&lt;user&gt;-&lt;project&gt;tensorflow-lite-float32-model.8.lite
-Nacher: trained_letter_S_F_Z_float32.lite
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Mit einem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Editor:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Editiere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Datei ei_image_classification_letter_S_F_Z_int8.py
-Hinter Zeile 12 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>einfügen</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve">sensor.set_vflip(True)      # Flips the image vertically
-sensor.set_hmirror(True)    # Mirrors the image horizontally
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ersetze</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> alle Vorkommen von labels.txt durch: labels_letter_S_F_Z.txt
-Ersetze alle Vorkommen von trained.tflite durch: trained_letter_S_F_Z_int8.tflite
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Speichern</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> nicht vergessen !!
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Kopiere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die geänderte Datei ei_image_classification_letter_S_F_Z_int8.py nach: ei_image_classification_letter_S_F_Z_float32.py
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Editiere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Datei ei_image_classification_letter_S_F_Z_float32.py
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ersetze</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> alle Vorkommen von trained_letter_S_F_Z_int8.tflite durch: trained_letter_S_F_Z_float32.lite</t>
-    </r>
-  </si>
-  <si>
     <t>Versorgungsspannung und digitale Pegel</t>
   </si>
   <si>
@@ -3604,912 +2748,13 @@
     <t>Verdrahtung der UART-Kommunikation zwischen OpenMV Cam und ESP32</t>
   </si>
   <si>
-    <t>Ausführung des Programms ei_image_classification_letter_S_F_Z_int8_serial_output.py</t>
-  </si>
-  <si>
     <t>Ausführung des Programms ESP32_UART_control_input_only.py</t>
   </si>
   <si>
     <t>OpenMV Cam ohne  IDE betreiben</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Schließe die OpenMV Cam über USB an den Computer an. Starte die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OpenMV IDE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Öffne das Programm ei_image_classification_letter_S_F_Z_int8_</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>serial_output</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.py.
-Das Programm ist eine Erweiterung des Programms, mit dem wir in den  letzten beiden Stunden gearbeitet haben. Das Programm macht eine Ausgabe, wenn Softmax  für ein Label einen Wert größer als den </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Schwellwert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 0,5 liefert. In der Ausgabe steht das erkannte </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Label</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> und die laufende </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nummer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> des Schnappschusses. Nur nach jedem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>10ten</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Schnappschuss wird eine Ausgabe gemacht, damit wir sie gut beobachten können. 
-Die Strings werden durch </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Leerzeichen</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> voneinander </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>getrennt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Das ist notwendig, damit der Empfänger Anfang und Ende der Strings erkennen kann. 
-print() schreibt die Ausgabe in das Serielle Terminal. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>uart.write()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> schreibt die Ausgabe auf den UART3. Während das Programm läuft, leuchtet  die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>LED blau.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-Der Schwellwert kann </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>geändert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> werden. Ebenso kann </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>geändert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> werden, nach wie vielen Schnappschüssen eine Ausgabe gemacht wird. 
-Führe nun das Programm aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. Fokussiere nun den Buchstaben S mit der Kamera und beobachte die Ausgaben am Seriellen Terminal. Bewege die Tafel mit dem Buchstaben hin und her und beobachte die Ausgabe im Seriellen Terminal.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Im </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Windows Datei-Explorer:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Schließe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Kamera an den Computer </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>an</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Das integrierte USB-Laufwerk wird als </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OpenMV D:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> angezeigt, 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Kopiere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Dateien vom Computer auf Laufwerk D: 
-ei_image_classification_letter_S_F_Z_float32.py
-ei_image_classification_letter_S_F_Z_int8.py
-labels_letter_S_F_Z.txt
-trained_letter_S_F_Z_int8.tflite
-trained_letter_S_F_Z_float32.lite
-In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">OpenMV IDE </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>testen:</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-Öffne </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>die Datei: ei_image_classification_letter_S_F_Z_int8.py</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Führe nun das </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>KI-Modell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> aus, indem du die OpenMV IDE mit der Kamera </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>verbindest</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> auf die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wiedergabetaste</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> klickst. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Fokussiere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> nun den Buchstaben S mit der Kamera und beobachte die Ausgaben am </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Seriellen Terminal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Ändere Abstand und Winkel zum Buchstaben S. Dieses KI-Modell läuft mit ca. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>13 Frames per Second.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Stoppe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> das Skript und beobachte die Ausgabe. Im KI-Modell wird </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>softmax</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> für Mehrklassenvorhersagen verwendet. Die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Summe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> aller von softmax erzeugten Ausgaben </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ist 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 
-Mit dem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Speichern-Symbol </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">speicherst du die Ausgaben in einer Log-Datei auf deinem Computer. Mit dem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wischen-Symbol</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> löschst du die Ausgaben im Seriellen Terminal bevor du das KI-Model erneut ausführt. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wiederhole</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> den Test mit der Datei ei_image_classification_letter_S_F_Z_float32.py
-Dieses (große) Modell läuft mit ca.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 3 Frames per Second.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">In einer Anwendung wird die OpenMV Cam </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ohne IDE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> betrieben.  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Dupliziere</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> das Programm ei_image_classification_letter_S_F_Z_int8_serial_output.py mit dem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Windows Datei-Explorer </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">auf dem USB-Laufwerk der OpenMV Cam. Es wir als OpenMV D: angezeigt, 
-Lösche die Originaldatei main.py oder benenne sie um. 
-Benenne das </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Duplikat</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">main.py </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">um. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Trenne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die OpenMV Cam vom Computer. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Verbinde</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> den OpenMV VIN Pin mit dem ESP32 5V Pin der ESP32-Platine. Nun bootet die OpenMV Cam und schreibt die Ausgaben auf den UART3. Während das Programm läuft, leuchtet  die LED blau. 
-Beobachte die Ausgaben in der ESP32 Shell.
-</t>
-    </r>
-  </si>
-  <si>
     <t>Verdrahtung der parallelen Kommunikation zwischen OpenMV Cam und ESP32</t>
-  </si>
-  <si>
-    <t>Ausführung des Programms ei_image_classification_letter_S_F_Z_int8_parallel_output.py</t>
   </si>
   <si>
     <t>Ausführung des Programms ESP32_parallel_input.py</t>
@@ -4546,120 +2791,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Schließe die OpenMV Cam über USB an den Computer an. Starte die OpenMV IDE. Öffne das Programm ei_image_classification_letter_S_F_Z_int8_parallel_output.py. 
-Das Programm ist eine Erweiterung des Programms, mit dem wir in den  letzten beiden Stunden gearbeitet haben. Das Programm macht eine Ausgabe, wenn Softmax  für ein Label einen Wert größer als den </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Schwellwert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 0,5 liefert. In der Ausgabe steht das erkannte Label und die laufende Nummer des Schnappschusses. Nur nach jedem </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>10ten</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Schnappschuss wird eine Ausgabe gemacht, damit wir sie gut beobachten können. 
-print() schreibt die Ausgabe in das Serielle Terminal. Das Programm macht aus dem Label String einen 2 Bit Code, der als </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Status der parallelen Output Pins </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">ausgegeben wird. Während das Programm läuft, leuchtet  die LED blau. 
-Der Schwellwert kann </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>geändert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> werden. Ebenso kann </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>geändert</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> werden, nach wie vielen Schnappschüssen eine Ausgabe gemacht wird.
-Führe nun das Programm aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. Fokussiere nun den Buchstaben S mit der Kamera und beobachte die Ausgaben am Seriellen Terminal. Bewege die Tafel mit dem Buchstaben hin und her und beobachte die Ausgabe im Seriellen Terminal.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Schließe die ESP32-Platine über den zweiten USB-Anschluss an den Computer an. Starte die </t>
     </r>
     <r>
@@ -4939,294 +3070,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OpenMV IDE:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Extras/ Datensatzeditor/ Export/ In Edge Impulse hochladen/ Projekt wählen/ Trainingsdaten 80% Testdaten 20% -&gt; 120 Dateien hinzugefügt
-In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Edge Impulse:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Öffne dein Projekt und navigiere zu </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Data Acquisition“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Du siehst, dass die </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bilder</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> hochgeladen und entsprechend den von Ihnen erstellten Klassen </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>gelabelt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> wurden. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Die Frage: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Are you building an object detection project" muss mit NO beantwortet werden. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wenn du das nicht tut, löscht Edge Impuls die Labels</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Abhilfe: Du</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> kannst über Project info/ Project info/ Labeling method wieder "One label per data item" einstellen. 
-Mit dem Data Acquisition Tool kannst du die Bildbeispiele durchsuchen und jene entfernen, die du für das Training als nicht wertvoll erachtest (z. B. wenn eines der Bilder zu unscharf ist). 
-Wenn du mit den Datensamples zufrieden sind, kannst du mit der Gestaltung deines Impulses fortfahren. Ein Impuls ist – kurz gesagt s– ein Rezept, anhand dessen das Modell trainiert wird. Er definiert Aktionen, die auf Ihre Eingabedaten angewendet werden, um diese für das maschinelle Lernen besser geeignet zu machen, sowie einen Lernblock, der den Algorithmus für die Klassifizierung festlegt. Navigiere im Menü unter </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">„Impulse Design“ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>zu</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> „Create Impulse“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> und füge sowohl einen </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Image Processing Block</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> als auch einen </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Transfer Learning Block</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> hinzu. Klicke auf </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Save Impulse“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, um die angepassten Einstellungen zu übernehmen.
-(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Verbinde die OpenMV-Kamera mithilfe eines </t>
     </r>
     <r>
@@ -5759,162 +3602,6 @@
       </rPr>
       <t xml:space="preserve"> Quantisierungsfehler wirken sich bei Netzwerken, die bereits an ihrer Kapazitätsgrenze arbeiten – d. h. bei denen jeder einzelne Parameter von entscheidender Bedeutung ist –, besonders gravierend aus. Wenn du dem Netzwerk einige zusätzliche Neuronen oder Schichten hinzufügst, wirst du möglicherweise feststellen, dass sich das Problem dadurch deutlich abschwächt.
 (https://docs.edgeimpulse.com/knowledge/guides/increasing-model-performance)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">In </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Edge Impulse: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Das ML-Modell ist trainiert und bereits für den Einsatz auf Mikrocontrollern optimiert. Dies erfolgt automatisch im Hintergrund durch Quantisierung. Dabei handelt es sich um einen Prozess, bei dem der Wertebereich der Zahlen innerhalb der Machine-Learning-Modelle eingeschränkt wird, um die Leistung zu steigern – unter Inkaufnahme eines geringfügigen Genauigkeitsverlusts.
-Wechsle im Menü zum Bereich </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Deployment“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, wähle unter </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Configure your deployment“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> die Option </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„OpenMV library“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> aus und klicke auf </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>„Build“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Dadurch wird eine </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bibliothek</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> erstellt, die deinen Impuls auf der OpenMV Cam ausführt. Entpacke die Datei, sobald der Download abgeschlossen ist. Der Download sollte automatisch starten. 
-(https://docs.arduino.cc/tutorials/nicla-vision/image-classification
-Die ZIP-Datei enthält nur das int8-Modell. So erhältst du das float32-Modell:
-Navigiere zu </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Dashboard/ Download block output. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Klicke auf das Schloss-Symbol neben TensorFlow Lite (float32), um den Download zu starten. </t>
     </r>
   </si>
   <si>
@@ -6639,12 +4326,728 @@
       <t xml:space="preserve"> zurück. Wenn keine Farbe erkannt wird, gibt die Funktion eine ungültige Zahl zurück.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpenMV IDE:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Extras/ Datensatzeditor/ Export/ In Edge Impulse hochladen/ Projekt wählen/ Trainingsdaten 80% Testdaten 20% -&gt; 120 Dateien hinzugefügt
+In </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Edge Impulse:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Öffne dein Projekt und navigiere zu </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Data Acquisition“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Du siehst, dass die </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bilder</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hochgeladen und entsprechend den von Ihnen erstellten Klassen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gelabelt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> wurden. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Die Frage: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Are you building an object detection project" muss mit NO beantwortet werden. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wenn du das nicht tut, löscht Edge Impuls die Labels</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Abhilfe: Du</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> kannst über Project info/ Project info/ Labeling method wieder "One label per data item" einstellen. 
+Mit dem Data Acquisition Tool kannst du die Bildbeispiele durchsuchen und jene entfernen, die du für das Training als nicht wertvoll erachtest (z. B. wenn eines der Bilder zu unscharf ist). 
+Wenn du mit den Datensamples zufrieden sind, kannst du mit der Gestaltung deines Impulses fortfahren. Ein Impuls ist – kurz gesagt – ein Rezept, anhand dessen das Modell trainiert wird. Er definiert Aktionen, die auf Ihre Eingabedaten angewendet werden, um diese für das maschinelle Lernen besser geeignet zu machen, sowie einen Lernblock, der den Algorithmus für die Klassifizierung festlegt. Navigiere im Menü unter </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">„Impulse Design“ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>zu</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> „Create Impulse“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> und füge sowohl einen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Image Processing Block</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> als auch einen </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Transfer Learning Block</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hinzu. Klicke auf </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Save Impulse“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, um die angepassten Einstellungen zu übernehmen.
+(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Edge Impulse:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In diesem Schritt passt du die Bildeinstellungen an und generierst die Merkmale aus den Eingabedaten. Merkmale sind eindeutige Eigenschaften, die vom Klassifizierungsalgorithmus verwendet werden, um die Objekte zu erkennen. (...) Navigieren im Menü unter „Impulse Design“ zum Punkt </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Image“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Stelle die Farbtiefe auf „RGB“ ein und </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>speichere die Parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+Klicke anschließend auf </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Generate Features“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Der Analysevorgang wird – abhängig von der Anzahl der hochgeladenen Bilder – einige Zeit in Anspruch nehmen.
+Sobald er abgeschlossen ist, kannst du die Ergebnisse begutachten. Im Feature Explorer siehst du eine Visualisierung der Merkmale. Du kannst erkennen, dass
+einige Buchstaben  (Punkte verschiedener Farbe) nur schwer voneinander zu unterscheiden sind, weil sich einige Datenpunkte in unmittelbarer Nähe zueinander befinden. Gibt es einen Buchstaben, der sich leichter abgrenzen lässt? (...)
+(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Edge Impulse: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Das ML-Modell ist trainiert und bereits für den Einsatz auf Mikrocontrollern optimiert. Dies erfolgt automatisch im Hintergrund durch Quantisierung. Dabei handelt es sich um einen Prozess, bei dem der Wertebereich der Zahlen innerhalb der Machine-Learning-Modelle eingeschränkt wird, um die Leistung zu steigern – unter Inkaufnahme eines geringfügigen Genauigkeitsverlusts.
+Wechsle im Menü zum Bereich </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Deployment“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, wähle unter </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Configure your deployment“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> die Option </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„OpenMV library“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> aus und klicke auf </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„Build“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Dadurch wird eine </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bibliothek</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> erstellt, die deinen Impuls auf der OpenMV Cam ausführt. Entpacke die Datei, sobald der Download abgeschlossen ist. Der Download sollte automatisch starten. 
+(https://docs.arduino.cc/tutorials/nicla-vision/image-classification
+Die ZIP-Datei enthält nur das int8-Modell. So erhältst du das float32-Modell:
+Navigiere zu </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Dashboard/ Download block output. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Klicke auf das Download-Symbol neben TensorFlow Lite (float32), um den Download zu starten. </t>
+    </r>
+  </si>
+  <si>
+    <t>In Netron.app:
+Öffne die Datei: trained_phi_psi_omega_int8.tflite
+Input und Output anschauen, int8, Dimensionen, Softmax
+Öffne die Datei: trained_phi_psi_omega_float32.lite
+Input und Output anschauen, float32, Dimensionen, Softmax</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In Edge Impulse: Benutzername, E-Mail-Adresse, Passwort (merken !!), Bedingungen zustimmen, E-Mail empfangen, Account aktivieren -&gt; Welcome 
+Create New Project, Name eingeben, Personal, Create New Project. 
+Target OpenMV H7 Plus auswählen
+Wenn später beim Hochladen der Daten nach Edge Impuls ein Authentifizierungs-Fehler gemeldet wird:  Keys/ Add new API key: Development Key Warnung ignorieren
+In OpenMV IDE: Extras/ Datensatzeditor/ Neuer Datensatz: Neuen
+ Ordner Phi_Psi_Omega erstellen und auswählen
+Bearbeite das ereits geöffnete Bildaufnahmeskript:
+Die Kamera steht auf dem Kopf. Füge deshalb hinter Zeile 12 ein: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>csi0.vflip(True) # Flips the image vertically</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>csi0.hmirror(True) # Mirrors the image horizontally</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Wir </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>beginnen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mit dem Buchstaben Omega, weil die OpenMV IDE die Ordner alphabetisch geordnet anzeigt. In der Werkzeugleiste: Klicke auf das Symbol Neuer Klassenordner/ letter_Omega erstellen. Führe nun das Bildaufnahmeskript aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. 
+Fokussiere den Buchstaben Omega mit der Kamera und klicke auf das Symbol Daten erfassen, um ein Bild davon aufzunehmen. Wiederhole dies 30x. Ändere Abstand und Winkel zwischen den Aufnahmen. 
+Ebenso: In der Werkzeugleiste ... letter_Phi ... Buchstabe Phi
+Ebenso: In der Werkzeugleiste ... letter_Psi ... Buchstabe Psi
+Ebenso: In der Werkzeugleiste ... unknown ... Buchstabe U oder leere Tafel
+(https://docs.arduino.cc/tutorials/nicla-vision/image-classification/)
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Im Windows Datei-Explorer: 
+Schließe die Kamera an den Computer an. Das integrierte USB-Laufwerk wird als OpenMV D: angezeigt, 
+Kopiere die Dateien vom Computer auf Laufwerk D: 
+ei_image_classification_phi_psi_omega_float32.py
+ei_image_classification_phi_psi_omega_int8.py
+labels_phi_psi_omega.txt
+trained_phi_psi_omega_int8.tflite
+trained_phi_psi_omega_float32.lite
+In OpenMV IDE testen: 
+Öffne die Datei: ei_image_classification_phi_psi_omega_int8.py
+Führe nun das KI-Modell aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. 
+Fokussiere nun den Buchstaben Phi mit der Kamera und beobachte die Ausgaben am Seriellen Terminal. Ändere Abstand und Winkel zum Buchstaben Phi. Dieses KI-Modell läuft mit ca. 13 Frames per Second. 
+Stoppe das Skript und beobachte die Ausgabe. Im KI-Modell wird softmax für Mehrklassenvorhersagen verwendet. Die Summe aller von softmax erzeugten Ausgaben ist 1. 
+Mit dem Speichern-Symbol speicherst du die Ausgaben in einer Log-Datei auf deinem Computer. Mit dem Wischen-Symbol löschst du die Ausgaben im Seriellen Terminal bevor du das KI-Model erneut ausführt. 
+Wiederhole den Test mit der Datei ei_image_classification_phi_psi_omega_float32.py
+Dieses (große) Modell läuft mit ca. 3 Frames per Second.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In einer Anwendung wird die OpenMV Cam ohne IDE betrieben.  
+Dupliziere das Programm ei_image_classification_phi_psi_omega_int8_serial_output.py mit dem Windows Datei-Explorer auf dem USB-Laufwerk der OpenMV Cam. Es wir als OpenMV D: angezeigt, 
+Lösche die Originaldatei main.py oder benenne sie um. 
+Benenne das Duplikat in main.py um. 
+Trenne die OpenMV Cam vom Computer. 
+Verbinde den OpenMV VIN Pin mit dem ESP32 5V Pin der ESP32-Platine. Nun bootet die OpenMV Cam und schreibt die Ausgaben auf den UART3. Während das Programm läuft, leuchtet  die LED blau. 
+Beobachte die Ausgaben in der ESP32 Shell.
+</t>
+  </si>
+  <si>
+    <t>Ausführung des Programms ei_image_classification_phi_psi_omega_int8_parallel_output.py</t>
+  </si>
+  <si>
+    <t>Schließe die OpenMV Cam über USB an den Computer an. Starte die OpenMV IDE. Öffne das Programm ei_image_classification_phi_psi_omega_int8_parallel_output.py. 
+Das Programm ist eine Erweiterung des Programms, mit dem wir in den  letzten beiden Stunden gearbeitet haben. Das Programm macht eine Ausgabe, wenn Softmax  für ein Label einen Wert größer als den Schwellwert 0,5 liefert. In der Ausgabe steht das erkannte Label und die laufende Nummer des Schnappschusses. Nur nach jedem 10ten Schnappschuss wird eine Ausgabe gemacht, damit wir sie gut beobachten können. 
+print() schreibt die Ausgabe in das Serielle Terminal. Das Programm macht aus dem Label String einen 2 Bit Code, der als Status der parallelen Output Pins ausgegeben wird. Während das Programm läuft, leuchtet  die LED blau. 
+Der Schwellwert kann geändert werden. Ebenso kann geändert werden, nach wie vielen Schnappschüssen eine Ausgabe gemacht wird.
+Führe nun das Programm aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. Fokussiere nun den Buchstaben S mit der Kamera und beobachte die Ausgaben am Seriellen Terminal. Bewege die Tafel mit dem Buchstaben hin und her und beobachte die Ausgabe im Seriellen Terminal.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Im Windows Datei-Explorer: 
+Entpacke die Datei ei-&lt;user&gt;-&lt;project&gt;-openmv-v-&lt;number&gt;-impulse-#1.zip
+Benenne die Dateien um:
+Vorher: trained.tflite  Nachher: trained_phi_psi_omega_int8.tflite
+Vorher: labels.txt         Nachher: labels_phi_psi_omega.txt
+Vorher: ei_image_classification.py 
+Nacher: ei_image_classification_phi_psi_omega_int8.py
+Vorher: ei-&lt;user&gt;-&lt;project&gt;tensorflow-lite-float32-model.8.lite
+Nacher: trained_phi_psi_omega_float32.lite
+Mit einem Editor: 
+Editiere die Datei ei_image_classification_phi_psi_omega_int8.py
+Hinter Zeile 12 einfügen: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">sensor.set_vflip(True)      # Flips the image vertically
+sensor.set_hmirror(True)    # Mirrors the image horizontally
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ersetze alle Vorkommen von labels.txt durch: labels_phi_psi_omega.txt
+Ersetze alle Vorkommen von trained.tflite durch: trained_phi_psi_omega_int8.tflite
+Speichern nicht vergessen !!
+Kopiere die geänderte Datei ei_image_classification_phi_psi_omega_int8.py nach: ei_image_classification_phi_psi_omega_float32.py
+Editiere die Datei ei_image_classification_phi_psi_omega_float32.py
+Ersetze alle Vorkommen von trained_phi_psi_omega_int8.tflite durch: trained_phi_psi_omega_float32.lite</t>
+    </r>
+  </si>
+  <si>
+    <t>Schließe die OpenMV Cam über USB an den Computer an. Starte die OpenMV IDE. Öffne das Programm ei_image_classification_phi_psi_omega_int8_serial_output.py.
+Das Programm ist eine Erweiterung des Programms, mit dem wir in den  letzten beiden Stunden gearbeitet haben. Das Programm macht eine Ausgabe, wenn Softmax  für ein Label einen Wert größer als den Schwellwert 0,5 liefert. In der Ausgabe steht das erkannte Label und die laufende Nummer des Schnappschusses. Nur nach jedem 10ten Schnappschuss wird eine Ausgabe gemacht, damit wir sie gut beobachten können. 
+Die Strings werden durch Leerzeichen voneinander getrennt. Das ist notwendig, damit der Empfänger Anfang und Ende der Strings erkennen kann. 
+print() schreibt die Ausgabe in das Serielle Terminal. uart.write() schreibt die Ausgabe auf den UART3. Während das Programm läuft, leuchtet  die LED blau. 
+Der Schwellwert kann geändert werden. Ebenso kann geändert werden, nach wie vielen Schnappschüssen eine Ausgabe gemacht wird. 
+Führe nun das Programm aus, indem du die OpenMV IDE mit der Kamera verbindest auf die Wiedergabetaste klickst. Fokussiere nun den Buchstaben Phi mit der Kamera und beobachte die Ausgaben am Seriellen Terminal. Bewege die Tafel mit dem Buchstaben hin und her und beobachte die Ausgabe im Seriellen Terminal.</t>
+  </si>
+  <si>
+    <t>Ausführung des Programms ei_image_classification_phi_psi_omega_int8_serial_output.py</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6716,6 +5119,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -7203,7 +5612,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" ht="165" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="165" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -7218,7 +5627,7 @@
       </c>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:5" ht="240" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="240" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
@@ -7233,7 +5642,7 @@
       </c>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="1:5" ht="135" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="135" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
@@ -7248,7 +5657,7 @@
       </c>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:5" ht="105" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -7265,7 +5674,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="30" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
@@ -7280,7 +5689,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="180" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="180" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>0</v>
       </c>
@@ -7295,7 +5704,7 @@
       </c>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="1:5" ht="270" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="270" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>0</v>
       </c>
@@ -7306,11 +5715,11 @@
         <v>18</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:5" ht="375" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="375" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
@@ -7327,7 +5736,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="45" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="45" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
@@ -7344,7 +5753,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="30" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -7357,7 +5766,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" ht="195" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="195" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -7372,7 +5781,7 @@
       </c>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:5" ht="270" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="270" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -7387,7 +5796,7 @@
       </c>
       <c r="E15" s="6"/>
     </row>
-    <row r="16" spans="1:5" ht="150" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="150" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>23</v>
       </c>
@@ -7402,7 +5811,7 @@
       </c>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" spans="1:5" ht="165" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="165" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
@@ -7417,7 +5826,7 @@
       </c>
       <c r="E17" s="6"/>
     </row>
-    <row r="18" spans="1:5" ht="105" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>23</v>
       </c>
@@ -7434,7 +5843,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="240" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="240" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>23</v>
       </c>
@@ -7451,7 +5860,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="60" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="60" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
@@ -7468,7 +5877,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
@@ -7510,10 +5919,10 @@
         <v>56</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="343.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" ht="405" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -7521,10 +5930,10 @@
         <v>14</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>64</v>
@@ -7541,7 +5950,7 @@
         <v>55</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>64</v>
@@ -7558,7 +5967,7 @@
         <v>57</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>45</v>
@@ -7575,7 +5984,7 @@
         <v>58</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>45</v>
@@ -7606,7 +6015,7 @@
         <v>53</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -7639,13 +6048,13 @@
         <v>61</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="342" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="360" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -7656,13 +6065,13 @@
         <v>66</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="390" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="405" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
@@ -7673,7 +6082,7 @@
         <v>67</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>71</v>
@@ -7690,7 +6099,7 @@
         <v>72</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>45</v>
@@ -7704,12 +6113,12 @@
         <v>53</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:5" ht="180" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" ht="180" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>28</v>
       </c>
@@ -7717,14 +6126,14 @@
         <v>7</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E36" s="6"/>
     </row>
-    <row r="37" spans="1:5" ht="120" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" ht="120" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>28</v>
       </c>
@@ -7732,16 +6141,16 @@
         <v>7</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="255" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" ht="255" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>28</v>
       </c>
@@ -7749,14 +6158,14 @@
         <v>14</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" ht="135" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" ht="135" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>28</v>
       </c>
@@ -7764,14 +6173,14 @@
         <v>14</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E39" s="2"/>
     </row>
-    <row r="40" spans="1:5" ht="150" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" ht="150" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>28</v>
       </c>
@@ -7779,14 +6188,14 @@
         <v>14</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" ht="120" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" ht="120" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>28</v>
       </c>
@@ -7794,14 +6203,14 @@
         <v>14</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="E41" s="2"/>
     </row>
-    <row r="42" spans="1:5" ht="240" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" ht="240" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>28</v>
       </c>
@@ -7809,16 +6218,16 @@
         <v>14</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="360" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" ht="360" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>28</v>
       </c>
@@ -7826,16 +6235,16 @@
         <v>7</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>29</v>
       </c>
@@ -7856,10 +6265,10 @@
         <v>7</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>45</v>
@@ -7873,16 +6282,16 @@
         <v>14</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="300" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" ht="315" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>29</v>
       </c>
@@ -7890,10 +6299,10 @@
         <v>14</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>101</v>
+        <v>136</v>
       </c>
       <c r="E47" s="2"/>
     </row>
@@ -7905,13 +6314,13 @@
         <v>14</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="E48" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="240" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -7922,10 +6331,10 @@
         <v>14</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>64</v>
@@ -7939,10 +6348,10 @@
         <v>14</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>45</v>
@@ -7956,10 +6365,10 @@
         <v>14</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>105</v>
+        <v>133</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="E51" s="2"/>
     </row>
@@ -7971,142 +6380,142 @@
         <v>14</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>53</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="1:5" ht="60" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" ht="60" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="E54" s="10"/>
     </row>
-    <row r="55" spans="1:5" ht="150" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" ht="150" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E55" s="10"/>
     </row>
-    <row r="56" spans="1:5" ht="105" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" ht="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E56" s="10"/>
     </row>
-    <row r="57" spans="1:5" ht="315" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" ht="315" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="339" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" ht="339" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="105" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" ht="105" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="409.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" ht="409.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="E60" s="11" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A61" s="12"/>
       <c r="B61" s="12"/>
       <c r="C61" s="12"/>

</xml_diff>